<commit_message>
revocup: rebuild deck math on real Shopify orders + sessions (19 slides), add sessions data to acquisition model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/revocup/acquisition-model.xlsx
+++ b/decks/revocup/acquisition-model.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -139,6 +139,10 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -542,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -651,12 +655,19 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Cost per click and conversion rate are illustrative. Conversion rate is the biggest unknown: the export has orders but no sessions.</t>
+          <t>Cost per click is illustrative. Today the store converts 0.82% of human sessions (Shopify Analytics, Oct 2025 to Sep 2026); the 1.5% default is a post-fix target, not a measurement.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Cost of goods is not entered in Shopify, so margin cannot be read from the store yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Sample is small (134 customers; 61 with a full year of history). Paid-social buyers may reorder less than today's mostly word-of-mouth buyers, so the Base case uses out-of-state customers and Conservative cuts that by 30%.</t>
         </is>
@@ -776,7 +787,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Unknown. Needs the Shopify sessions report</t>
+          <t>Target after store fixes. Today the store converts 0.82% (Shopify Analytics, Oct 2025 to Sep 2026)</t>
         </is>
       </c>
     </row>
@@ -1048,22 +1059,22 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>0.0026</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="C4" s="21" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="F4" s="21" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="G4" s="21" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="5">
@@ -1265,7 +1276,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>0.26% is what the store converts today if Habte's 8,000 monthly visits are right (about 20 orders a month). Confirm with the sessions report.</t>
+          <t>0.82% is what the store converted over the last 12 months (human sessions, Shopify Analytics). The store setup sprint aims to lift it before ads scale.</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2452,6 +2463,317 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Store traffic · human sessions (Shopify Analytics, bots excluded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Added to cart</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>Completed checkout</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Conversion rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="32" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="n">
+        <v>2155</v>
+      </c>
+      <c r="C61" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D61" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E61" s="33">
+        <f>IF(B61=0,0,D61/B61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="32" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C62" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="D62" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E62" s="33">
+        <f>IF(B62=0,0,D62/B62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="32" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="n">
+        <v>2131</v>
+      </c>
+      <c r="C63" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="D63" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="E63" s="33">
+        <f>IF(B63=0,0,D63/B63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="32" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C64" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D64" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E64" s="33">
+        <f>IF(B64=0,0,D64/B64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="32" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="n">
+        <v>1762</v>
+      </c>
+      <c r="C65" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="D65" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E65" s="33">
+        <f>IF(B65=0,0,D65/B65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="32" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B66" s="10" t="n">
+        <v>2121</v>
+      </c>
+      <c r="C66" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="D66" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="E66" s="33">
+        <f>IF(B66=0,0,D66/B66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="32" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="n">
+        <v>2107</v>
+      </c>
+      <c r="C67" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D67" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="E67" s="33">
+        <f>IF(B67=0,0,D67/B67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="32" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>2271</v>
+      </c>
+      <c r="C68" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D68" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E68" s="33">
+        <f>IF(B68=0,0,D68/B68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="32" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="n">
+        <v>2238</v>
+      </c>
+      <c r="C69" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="D69" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="E69" s="33">
+        <f>IF(B69=0,0,D69/B69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="32" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="n">
+        <v>2149</v>
+      </c>
+      <c r="C70" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="D70" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="E70" s="33">
+        <f>IF(B70=0,0,D70/B70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="32" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="n">
+        <v>2084</v>
+      </c>
+      <c r="C71" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D71" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="E71" s="33">
+        <f>IF(B71=0,0,D71/B71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="32" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="n">
+        <v>2335</v>
+      </c>
+      <c r="C72" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="D72" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E72" s="33">
+        <f>IF(B72=0,0,D72/B72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>12-month total</t>
+        </is>
+      </c>
+      <c r="B73" s="34">
+        <f>SUM(B61:B72)</f>
+        <v/>
+      </c>
+      <c r="C73" s="34">
+        <f>SUM(C61:C72)</f>
+        <v/>
+      </c>
+      <c r="D73" s="34">
+        <f>SUM(D61:D72)</f>
+        <v/>
+      </c>
+      <c r="E73" s="35">
+        <f>IF(B73=0,0,D73/B73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>By source, Oct 2025 to Oct 13 2026, human sessions: Direct 16,250 at 0.63%; Search 9,671 at 1.11%; Social 235 at 0%. Bots added about 6,900 more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>About 1.5% of sessions add to cart; about 62% of sessions that reach checkout complete it. The leak is before the cart.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
revocup: QA fixes (new-customer conversion 0.3% baseline, 0.3/1/2% scenarios, brand mentions instead of AI Visibility, model formula fix)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/revocup/acquisition-model.xlsx
+++ b/decks/revocup/acquisition-model.xlsx
@@ -655,7 +655,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Cost per click is illustrative. Today the store converts 0.82% of human sessions (Shopify Analytics, Oct 2025 to Sep 2026); the 1.5% default is a post-fix target, not a measurement.</t>
+          <t>Cost per click is illustrative. Today the store converts 0.82% of human sessions (Shopify Analytics, Oct 2025 to Sep 2026); only about 0.3% of visits bring in a NEW customer. The 1% default is a post-fix target, not a measurement.</t>
         </is>
       </c>
     </row>
@@ -779,15 +779,15 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Site conversion rate, paid visitors</t>
+          <t>Site conversion rate, first-time paid visitors</t>
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Target after store fixes. Today the store converts 0.82% (Shopify Analytics, Oct 2025 to Sep 2026)</t>
+          <t>Target after store fixes. Today about 0.3% of visits bring in a new customer (0.82% counting repeat orders)</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="B15" s="16">
-        <f>ROUND('Shopify data'!E32*0.7,2)</f>
+        <f>ROUND('Shopify data'!D32*0.7,2)</f>
         <v/>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1059,22 +1059,22 @@
         </is>
       </c>
       <c r="B4" s="21" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.003</v>
       </c>
       <c r="C4" s="21" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D4" s="21" t="n">
         <v>0.01</v>
       </c>
-      <c r="D4" s="21" t="n">
+      <c r="E4" s="21" t="n">
         <v>0.015</v>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="F4" s="21" t="n">
         <v>0.02</v>
       </c>
-      <c r="F4" s="21" t="n">
+      <c r="G4" s="21" t="n">
         <v>0.025</v>
-      </c>
-      <c r="G4" s="21" t="n">
-        <v>0.03</v>
       </c>
     </row>
     <row r="5">
@@ -1276,7 +1276,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>0.82% is what the store converted over the last 12 months (human sessions, Shopify Analytics). The store setup sprint aims to lift it before ads scale.</t>
+          <t>0.3% is the rate at which a visit brings in a NEW customer today (73 new customers over 25,519 human sessions, last 12 months). All orders over sessions is 0.82%, but about two-thirds of orders are repeat buyers, and ad visitors are all first-time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
revocup: Oct 15 call updates (60% margin, $1,750 Meta+Google, flexible ad budget, Proof Syrup case study, path to scale, team/UGC; 25 slides)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/revocup/acquisition-model.xlsx
+++ b/decks/revocup/acquisition-model.xlsx
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared by EmberTribe, October 14, 2026. Internal working model for the 90-day paid social test.</t>
+          <t>Prepared by EmberTribe, updated October 15, 2026. Internal working model for the 90-day paid social test.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Gross margin (70%) is an assumption from the Oct 12 call until Revocup confirms cost per bag.</t>
+          <t>Gross margin (60%) is Habte's estimate for roasted beans from the Oct 15 call; cost of goods is not entered in Shopify.</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Habte, Oct 12 call</t>
+          <t>Habte, Oct 12 call; Oct 15: flexible, from $3,000</t>
         </is>
       </c>
     </row>
@@ -753,11 +753,11 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Assumption from the call. Replace with real cost per bag</t>
+          <t>Habte, Oct 15 call: about 60% on roasted beans, possibly lower</t>
         </is>
       </c>
     </row>
@@ -798,26 +798,26 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>4500</v>
+        <v>1750</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Rate card: Meta management $2,500 + email/SMS $2,000</t>
+          <t>Meta + Google management, discounted Oct 15 (standard $2,500 one channel). Add $2,000 for email/SMS campaigns</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>One-time store setup</t>
+          <t>One-time site redesign</t>
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1250</v>
+        <v>5000</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Store setup sprint, month 1</t>
+          <t>Elite Launch at $5,000 with a 90-day paid media commitment signed by Oct 31, 2026 ($9,999 alone)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
revocup: QA fixes (Proof Syrup wording to match case study, scale slide shows fees and 1% case, Google in tracking/timeline)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/revocup/acquisition-model.xlsx
+++ b/decks/revocup/acquisition-model.xlsx
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared by EmberTribe, updated October 15, 2026. Internal working model for the 90-day paid social test.</t>
+          <t>Prepared by EmberTribe, updated October 15, 2026. Internal working model for the 90-day paid media test (Meta and Google).</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Cost per click (Meta)</t>
+          <t>Cost per click (Meta and Google, blended)</t>
         </is>
       </c>
       <c r="B7" s="12" t="n">

</xml_diff>